<commit_message>
Edição de indicadores, recursos e revisores de quick win; alteração na medição com motivo
Tela para editar indicadores, recursos e revisores de um quick win já
criado. Depois de iniciada a medição, mudar indicador, ponto de partida ou
janela exige motivo, fica na auditoria e em registro próprio, e o relatório
de resultados (PDF e XLSX) mostra que houve alteração. Teste de desmontagem
deixa de derrubar o arquivo quando o drop encerra conexões abertas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015mqTFtP1jGUbbpXgao4Nue
</commit_message>
<xml_diff>
--- a/docs/fase-3b/relatorios-construtora/resultados-quick-wins.xlsx
+++ b/docs/fase-3b/relatorios-construtora/resultados-quick-wins.xlsx
@@ -6,15 +6,16 @@
   <sheets>
     <sheet sheetId="1" name="Quick wins" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Antes × depois" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Valores registrados" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Sobre" state="visible" r:id="rId7"/>
+    <sheet sheetId="3" name="Alterações na medição" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Valores registrados" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Sobre" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="144">
   <si>
     <t>Quick win</t>
   </si>
@@ -40,6 +41,9 @@
     <t>Avisos das janelas</t>
   </si>
   <si>
+    <t>Alterações na medição</t>
+  </si>
+  <si>
     <t>Decisão</t>
   </si>
   <si>
@@ -76,6 +80,9 @@
     <t>Janelas com duração muito diferente: 92 dias no ponto de partida e 20 dias na medição. Compare por mês ou por item. Volume muito diferente: 360 cotações no ponto de partida e 80 cotações na medição. Compare por item.</t>
   </si>
   <si>
+    <t>2026-09-24 ponto de partida de Tempo por cotação conferida: 32 min (key.suprimentos@horizonte.com.br): O valor informado não contava a conferência da unidade; foi medido de novo.</t>
+  </si>
+  <si>
     <t>manter</t>
   </si>
   <si>
@@ -109,6 +116,9 @@
     <t>2026-10-01 a 2026-10-07 (7 dias)</t>
   </si>
   <si>
+    <t>nenhuma</t>
+  </si>
+  <si>
     <t>sem ponto de partida</t>
   </si>
   <si>
@@ -217,63 +227,90 @@
     <t>min</t>
   </si>
   <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>medido: medido de 2026-08-01 a 2026-08-31; método: cronometragem de 30 cotações</t>
+  </si>
+  <si>
+    <t>sem medição</t>
+  </si>
+  <si>
+    <t>sem medição depois</t>
+  </si>
+  <si>
+    <t>Ligações ao técnico por semana</t>
+  </si>
+  <si>
+    <t>ligações</t>
+  </si>
+  <si>
+    <t>Horas de leitura do diário por semana</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>medido: medido de 2026-08-01 a 2026-08-15; método: cronometragem de dois engenheiros</t>
+  </si>
+  <si>
+    <t>0,8</t>
+  </si>
+  <si>
+    <t>medido: medido de 2026-09-08 a 2026-09-22; método: cronometragem de dois engenheiros, com revisão</t>
+  </si>
+  <si>
+    <t>-3,2 (-80%)</t>
+  </si>
+  <si>
+    <t>57,6 h = (4 − 0.8) h × 18 semanas de canteiro na janela de medição</t>
+  </si>
+  <si>
+    <t>Resumos aprovados sem edição</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>66,7</t>
+  </si>
+  <si>
+    <t>automático: média das execuções de 2026-09-05 a 2026-09-24 (4 concluídas)</t>
+  </si>
+  <si>
     <t>25</t>
   </si>
   <si>
-    <t>informado: informado por Coordenação de suprimentos em 2026-09-24</t>
-  </si>
-  <si>
-    <t>sem medição</t>
-  </si>
-  <si>
-    <t>sem medição depois</t>
-  </si>
-  <si>
-    <t>Ligações ao técnico por semana</t>
-  </si>
-  <si>
-    <t>ligações</t>
-  </si>
-  <si>
-    <t>Horas de leitura do diário por semana</t>
-  </si>
-  <si>
-    <t>h</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>medido: medido de 2026-08-01 a 2026-08-15; método: cronometragem de dois engenheiros</t>
-  </si>
-  <si>
-    <t>0,8</t>
-  </si>
-  <si>
-    <t>medido: medido de 2026-09-08 a 2026-09-22; método: cronometragem de dois engenheiros, com revisão</t>
-  </si>
-  <si>
-    <t>-3,2 (-80%)</t>
-  </si>
-  <si>
-    <t>57,6 h = (4 − 0.8) h × 18 semanas de canteiro na janela de medição</t>
-  </si>
-  <si>
-    <t>Resumos aprovados sem edição</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>66,7</t>
-  </si>
-  <si>
-    <t>automático: média das execuções de 2026-09-05 a 2026-09-24 (4 concluídas)</t>
-  </si>
-  <si>
     <t>medido: medido de 2026-09-01 a 2026-09-07; método: registro de chamados do técnico</t>
   </si>
   <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>O que mudou</t>
+  </si>
+  <si>
+    <t>Motivo</t>
+  </si>
+  <si>
+    <t>Quem</t>
+  </si>
+  <si>
+    <t>2026-09-24</t>
+  </si>
+  <si>
+    <t>em medição</t>
+  </si>
+  <si>
+    <t>ponto de partida de Tempo por cotação conferida: 32 min</t>
+  </si>
+  <si>
+    <t>O valor informado não contava a conferência da unidade; foi medido de novo.</t>
+  </si>
+  <si>
     <t>quickWin</t>
   </si>
   <si>
@@ -334,7 +371,19 @@
     <t/>
   </si>
   <si>
-    <t>2026-09-24T15:13:54.731Z</t>
+    <t>2026-09-24T17:23:19.565Z</t>
+  </si>
+  <si>
+    <t>tempo_por_cotacao</t>
+  </si>
+  <si>
+    <t>informado</t>
+  </si>
+  <si>
+    <t>Coordenação de suprimentos</t>
+  </si>
+  <si>
+    <t>2026-09-24T17:23:19.580Z</t>
   </si>
   <si>
     <t>depois</t>
@@ -346,34 +395,28 @@
     <t>2026-09-30</t>
   </si>
   <si>
-    <t>2026-09-24T15:13:54.748Z</t>
-  </si>
-  <si>
-    <t>tempo_por_cotacao</t>
-  </si>
-  <si>
-    <t>informado</t>
-  </si>
-  <si>
-    <t>Coordenação de suprimentos</t>
-  </si>
-  <si>
-    <t>2026-09-24T15:13:54.762Z</t>
+    <t>2026-09-24T17:23:20.260Z</t>
+  </si>
+  <si>
+    <t>2026-08-01</t>
+  </si>
+  <si>
+    <t>cronometragem de 30 cotações</t>
+  </si>
+  <si>
+    <t>2026-09-24T17:23:20.273Z</t>
   </si>
   <si>
     <t>horas_leitura</t>
   </si>
   <si>
-    <t>2026-08-01</t>
-  </si>
-  <si>
     <t>2026-08-15</t>
   </si>
   <si>
     <t>cronometragem de dois engenheiros</t>
   </si>
   <si>
-    <t>2026-09-24T15:13:54.794Z</t>
+    <t>2026-09-24T17:23:19.594Z</t>
   </si>
   <si>
     <t>2026-09-08</t>
@@ -385,7 +428,7 @@
     <t>cronometragem de dois engenheiros, com revisão</t>
   </si>
   <si>
-    <t>2026-09-24T15:13:54.811Z</t>
+    <t>2026-09-24T17:23:20.303Z</t>
   </si>
   <si>
     <t>ligacoes_tecnico</t>
@@ -397,7 +440,7 @@
     <t>registro de chamados do técnico</t>
   </si>
   <si>
-    <t>2026-09-24T15:13:54.778Z</t>
+    <t>2026-09-24T17:23:20.289Z</t>
   </si>
   <si>
     <t>Resultados dos quick wins: Construtora Horizonte (demonstração)</t>
@@ -784,7 +827,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="12" customWidth="1"/>
@@ -793,13 +836,14 @@
     <col min="6" max="6" width="28" customWidth="1"/>
     <col min="7" max="7" width="19" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="9" max="9" width="23" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -836,195 +880,213 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="D4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L4" t="s">
         <v>24</v>
       </c>
-      <c r="B3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="M4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>26</v>
       </c>
-      <c r="D3" t="s">
+      <c r="B5" t="s">
         <v>27</v>
       </c>
-      <c r="E3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" t="s">
         <v>29</v>
       </c>
-      <c r="G3" t="s">
+      <c r="E5" t="s">
         <v>30</v>
       </c>
-      <c r="H3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="F5" t="s">
         <v>31</v>
       </c>
-      <c r="L3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="G5" t="s">
         <v>32</v>
       </c>
-      <c r="B4" t="s">
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" t="s">
         <v>33</v>
       </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="J5" t="s">
+        <v>25</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L6" t="s">
         <v>34</v>
       </c>
-      <c r="E4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G4" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" t="s">
-        <v>38</v>
-      </c>
-      <c r="J4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" t="s">
-        <v>22</v>
-      </c>
-      <c r="L4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" t="s">
-        <v>23</v>
-      </c>
-      <c r="J5" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" t="s">
-        <v>22</v>
-      </c>
-      <c r="L5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6" t="s">
-        <v>43</v>
-      </c>
-      <c r="G6" t="s">
-        <v>44</v>
-      </c>
-      <c r="H6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J6" t="s">
-        <v>23</v>
-      </c>
-      <c r="K6" t="s">
-        <v>31</v>
-      </c>
-      <c r="L6" t="s">
-        <v>45</v>
+      <c r="M6" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1053,314 +1115,314 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="J2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="K2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
         <v>72</v>
       </c>
-      <c r="D4" t="s">
-        <v>72</v>
-      </c>
-      <c r="E4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" t="s">
-        <v>69</v>
-      </c>
       <c r="I4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="K4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="G5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="H5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="J5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="K5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="H6" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="I6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="K6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" t="s">
+        <v>89</v>
+      </c>
+      <c r="G7" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" t="s">
         <v>72</v>
       </c>
-      <c r="D7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F7" t="s">
-        <v>85</v>
-      </c>
-      <c r="G7" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" t="s">
-        <v>69</v>
-      </c>
       <c r="I7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J7" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="K8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H9" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="K9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1371,7 +1433,63 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="6" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="12" customWidth="1"/>
@@ -1381,289 +1499,330 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="C2" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="D2">
         <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F2" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="G2" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="H2" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="I2" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="J2" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="K2" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="L2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M2" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="C3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="F3" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="G3" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="H3" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="I3" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="J3" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="K3" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="L3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M3" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>111</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="D4">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="F4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G4" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="H4" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="I4" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="J4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="K4" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="L4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M4" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D5">
         <v>32</v>
       </c>
-      <c r="B5" t="s">
+      <c r="E5" t="s">
+        <v>69</v>
+      </c>
+      <c r="F5" t="s">
+        <v>113</v>
+      </c>
+      <c r="G5" t="s">
+        <v>127</v>
+      </c>
+      <c r="H5" t="s">
         <v>115</v>
       </c>
-      <c r="C5" t="s">
-        <v>100</v>
-      </c>
-      <c r="D5">
-        <v>4</v>
-      </c>
-      <c r="E5" t="s">
-        <v>74</v>
-      </c>
-      <c r="F5" t="s">
-        <v>101</v>
-      </c>
-      <c r="G5" t="s">
-        <v>116</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
+        <v>128</v>
+      </c>
+      <c r="J5" t="s">
         <v>117</v>
       </c>
-      <c r="I5" t="s">
-        <v>118</v>
-      </c>
-      <c r="J5" t="s">
-        <v>105</v>
-      </c>
       <c r="K5" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="L5" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="M5" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="C6" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D6">
-        <v>0.8</v>
+        <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F6" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="G6" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H6" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="I6" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="J6" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="K6" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="L6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="M6" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7">
+        <v>0.8</v>
+      </c>
+      <c r="E7" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" t="s">
+        <v>113</v>
+      </c>
+      <c r="G7" t="s">
+        <v>134</v>
+      </c>
+      <c r="H7" t="s">
+        <v>135</v>
+      </c>
+      <c r="I7" t="s">
+        <v>136</v>
+      </c>
+      <c r="J7" t="s">
+        <v>117</v>
+      </c>
+      <c r="K7" t="s">
+        <v>117</v>
+      </c>
+      <c r="L7" t="s">
+        <v>37</v>
+      </c>
+      <c r="M7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D8">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" t="s">
+        <v>113</v>
+      </c>
+      <c r="G8" t="s">
         <v>124</v>
       </c>
-      <c r="C7" t="s">
-        <v>100</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7" t="s">
-        <v>72</v>
-      </c>
-      <c r="F7" t="s">
-        <v>101</v>
-      </c>
-      <c r="G7" t="s">
-        <v>108</v>
-      </c>
-      <c r="H7" t="s">
-        <v>125</v>
-      </c>
-      <c r="I7" t="s">
-        <v>126</v>
-      </c>
-      <c r="J7" t="s">
-        <v>105</v>
-      </c>
-      <c r="K7" t="s">
-        <v>105</v>
-      </c>
-      <c r="L7" t="s">
-        <v>27</v>
-      </c>
-      <c r="M7" t="s">
-        <v>127</v>
+      <c r="H8" t="s">
+        <v>139</v>
+      </c>
+      <c r="I8" t="s">
+        <v>140</v>
+      </c>
+      <c r="J8" t="s">
+        <v>117</v>
+      </c>
+      <c r="K8" t="s">
+        <v>117</v>
+      </c>
+      <c r="L8" t="s">
+        <v>29</v>
+      </c>
+      <c r="M8" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -1672,7 +1831,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1682,12 +1841,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>